<commit_message>
v18 三通道改成按物理邻居 0.926 v19 两个序列，本地就低 v20 五折交叉 ，0.927 v21 resnet0.928 v22 mq model 0.925
</commit_message>
<xml_diff>
--- a/实验记录表.xlsx
+++ b/实验记录表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Kaggle\RSNA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C52480B-5337-4B9A-B5C6-6E9AE18274B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E237752-F197-4255-92A8-BDABAC44E71D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="55">
   <si>
     <t>版本</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -204,6 +204,45 @@
   </si>
   <si>
     <t>原图+ 增强的一起训练</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v18</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>三通道改成按物理距离选邻居</t>
+  </si>
+  <si>
+    <t>v19</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>最多两个序列，候选120 ， 窗口36</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>五折训练，验证集用分出来的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v21</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>backbone radimagenet resnte50 backbone lr 3e-4 imgsz224</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v22</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>mq model</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -539,11 +578,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.58203125" customWidth="1"/>
-    <col min="2" max="2" width="69.4140625" customWidth="1"/>
+    <col min="2" max="2" width="85.25" customWidth="1"/>
     <col min="3" max="3" width="24.9140625" customWidth="1"/>
     <col min="4" max="4" width="22.08203125" customWidth="1"/>
   </cols>
@@ -906,6 +945,88 @@
       <c r="D23" s="1">
         <v>0.90790000000000004</v>
       </c>
+      <c r="E23" s="1">
+        <v>0.92700000000000005</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="1">
+        <v>19</v>
+      </c>
+      <c r="D24" s="1">
+        <v>0.91173000000000004</v>
+      </c>
+      <c r="E24" s="1">
+        <v>0.92600000000000005</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" s="1">
+        <v>14</v>
+      </c>
+      <c r="D25" s="1">
+        <v>0.90400000000000003</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D26" s="1">
+        <v>0.90475000000000005</v>
+      </c>
+      <c r="E26" s="1">
+        <v>0.92600000000000005</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="1">
+        <v>18</v>
+      </c>
+      <c r="D27" s="1">
+        <v>0.90720000000000001</v>
+      </c>
+      <c r="E27" s="1">
+        <v>0.92800000000000005</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="1">
+        <v>19</v>
+      </c>
+      <c r="D28" s="1">
+        <v>0.91069999999999995</v>
+      </c>
+      <c r="E28" s="1">
+        <v>0.92500000000000004</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
v19最多两个序列，候选120，窗口36 本地0.904 v20五折训练0.926 v21 resnet 0.928 v22 mq model 0.925 v23 resnet 五折0.929 v24 千问微调
</commit_message>
<xml_diff>
--- a/实验记录表.xlsx
+++ b/实验记录表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Kaggle\RSNA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E237752-F197-4255-92A8-BDABAC44E71D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8457301B-F643-44F2-B310-7395EBFE2A2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="57">
   <si>
     <t>版本</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -243,6 +243,14 @@
   </si>
   <si>
     <t>mq model</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v23</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>resnet 五折</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -578,7 +586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.58203125" customWidth="1"/>
@@ -1028,6 +1036,18 @@
         <v>0.92500000000000004</v>
       </c>
     </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1">
+        <v>0.92900000000000005</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>